<commit_message>
register: v2.3 sweep over S007 — FEDIOL geography, ports exception, mengvoeder note
Verified S007 rule by rule against protocol v2.3: edibility, L5 on the animal
branch, and the conversion arithmetic were all already applied in the review
pass. The sweep found one further gap, present in both sources:

- the consolidated-table NACE 10.4 oil rows (C-279/C-280 in S091, C-464/C-465
  in S007) carried a Belgian FEDIOL figure at geography=Vlaanderen, the same
  "table title is not the definition" pattern as the sugar rows. Corrected to
  Belgie. They restate the FEDIOL totals exactly, so each pair is now
  cross-referenced for the reviewer to collapse.
- S091's four landing rows now invoke the sanctioned Belgian-ports exception
  by name, as S080's and S002's already did.

Mengvoeder: the reviewer's rejection of the S091 block is source-specific, not
a scope rule. Recorded as resolved in hub.md; S007's block stays captured.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/register/BIOLOOP_streams_and_sources.xlsx
+++ b/database/register/BIOLOOP_streams_and_sources.xlsx
@@ -28770,7 +28770,7 @@
       </c>
       <c r="U270" t="inlineStr">
         <is>
-          <t>aanlanding door Belgische vissersvaartuigen; 99% hoofdstromen</t>
+          <t>aanlanding door Belgische vissersvaartuigen; 99% hoofdstromen Bron schrijft "Belgische vissersvaartuigen"; alle Belgische vissershavens liggen in Vlaanderen, zodat het nationale en het Vlaamse cijfer samenvallen (gesanctioneerde uitzondering op de geography-regel).</t>
         </is>
       </c>
       <c r="V270" t="inlineStr">
@@ -28884,7 +28884,7 @@
       </c>
       <c r="U271" t="inlineStr">
         <is>
-          <t>aangeland door Belgische vissersvaartuigen</t>
+          <t>aangeland door Belgische vissersvaartuigen Bron schrijft "Belgische vissersvaartuigen"; alle Belgische vissershavens liggen in Vlaanderen, zodat het nationale en het Vlaamse cijfer samenvallen (gesanctioneerde uitzondering op de geography-regel).</t>
         </is>
       </c>
       <c r="V271" t="inlineStr">
@@ -28998,7 +28998,7 @@
       </c>
       <c r="U272" t="inlineStr">
         <is>
-          <t>aangeland door Belgische vissersvaartuigen</t>
+          <t>aangeland door Belgische vissersvaartuigen Bron schrijft "Belgische vissersvaartuigen"; alle Belgische vissershavens liggen in Vlaanderen, zodat het nationale en het Vlaamse cijfer samenvallen (gesanctioneerde uitzondering op de geography-regel).</t>
         </is>
       </c>
       <c r="V272" t="inlineStr">
@@ -29112,7 +29112,7 @@
       </c>
       <c r="U273" t="inlineStr">
         <is>
-          <t>aangeland door Belgische vissersvaartuigen</t>
+          <t>aangeland door Belgische vissersvaartuigen Bron schrijft "Belgische vissersvaartuigen"; alle Belgische vissershavens liggen in Vlaanderen, zodat het nationale en het Vlaamse cijfer samenvallen (gesanctioneerde uitzondering op de geography-regel).</t>
         </is>
       </c>
       <c r="V273" t="inlineStr">
@@ -29798,7 +29798,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>AGGREGAAT - Vervaardiging van plantaardige en dierlijke olien en vetten, productie hoofdstromen</t>
+          <t>AGGREGAAT - Vervaardiging van plantaardige en dierlijke olien en vetten, productie hoofdstromen (Belgisch FEDIOL-cijfer, door de bron in de Vlaamse tabel gezet)</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -29860,7 +29860,7 @@
       </c>
       <c r="U280" t="inlineStr">
         <is>
-          <t>geconsolideerde tabel voedingssector, kolom productie/hoofd; overgenomen uit Tabel 32 (FEDIOL, Belgie) maar hier als Vlaams cijfer gepresenteerd</t>
+          <t>geconsolideerde tabel voedingssector, kolom productie/hoofd; overgenomen uit Tabel 32 (FEDIOL, Belgie) maar hier als Vlaams cijfer gepresenteerd De tabeltitel zegt "Vlaamse voedingssector", maar de bron stelt zelf dat voor NACE 10.4 de FEDIOL-cijfers voor Belgie gebruikt zijn; de materiele dekking is dus Belgisch en geography staat daarom op Belgie.</t>
         </is>
       </c>
       <c r="V280" t="inlineStr">
@@ -29870,12 +29870,17 @@
       </c>
       <c r="W280" t="inlineStr">
         <is>
-          <t>Vlaanderen</t>
+          <t>Belgie</t>
         </is>
       </c>
       <c r="X280" t="inlineStr">
         <is>
           <t>read in PDF</t>
+        </is>
+      </c>
+      <c r="Z280" t="inlineStr">
+        <is>
+          <t>zelfde getal en zelfde dekking als C-329 (Tabel 32, FEDIOL Belgie, p.91) - dit is een herhaling van dat cijfer in de samenvattende tabel, geen onafhankelijke meting; de reviewer kan een van beide rijen laten vervallen</t>
         </is>
       </c>
     </row>
@@ -29897,7 +29902,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>AGGREGAAT - Vervaardiging van plantaardige en dierlijke olien en vetten, productie nevenstromen en productieresiduen</t>
+          <t>AGGREGAAT - Vervaardiging van plantaardige en dierlijke olien en vetten, productie nevenstromen en productieresiduen (Belgisch FEDIOL-cijfer, door de bron in de Vlaamse tabel gezet)</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -29959,7 +29964,7 @@
       </c>
       <c r="U281" t="inlineStr">
         <is>
-          <t>geconsolideerde tabel voedingssector, kolom productie/nev-res; overgenomen uit Tabel 33 (FEDIOL, Belgie) maar hier als Vlaams cijfer gepresenteerd</t>
+          <t>geconsolideerde tabel voedingssector, kolom productie/nev-res; overgenomen uit Tabel 33 (FEDIOL, Belgie) maar hier als Vlaams cijfer gepresenteerd De tabeltitel zegt "Vlaamse voedingssector", maar de bron stelt zelf dat voor NACE 10.4 de FEDIOL-cijfers voor Belgie gebruikt zijn; de materiele dekking is dus Belgisch en geography staat daarom op Belgie.</t>
         </is>
       </c>
       <c r="V281" t="inlineStr">
@@ -29969,12 +29974,17 @@
       </c>
       <c r="W281" t="inlineStr">
         <is>
-          <t>Vlaanderen</t>
+          <t>Belgie</t>
         </is>
       </c>
       <c r="X281" t="inlineStr">
         <is>
           <t>read in PDF</t>
+        </is>
+      </c>
+      <c r="Z281" t="inlineStr">
+        <is>
+          <t>zelfde getal en zelfde dekking als C-335 (Tabel 33, FEDIOL Belgie, p.91) - dit is een herhaling van dat cijfer in de samenvattende tabel, geen onafhankelijke meting; de reviewer kan een van beide rijen laten vervallen</t>
         </is>
       </c>
     </row>
@@ -35235,7 +35245,7 @@
       </c>
       <c r="Z330" t="inlineStr">
         <is>
-          <t>hetzelfde getal staat als Vlaams cijfer in Tabel 26 (p.76) - zie de anomalienota</t>
+          <t>hetzelfde getal staat in Tabel 26 (p.76) in de kolom van de Vlaamse voedingssector - zie C-279, dat nu eveneens geography Belgie draagt; '504 kton voor Belgie' ook in tekst p.90 en p.4</t>
         </is>
       </c>
     </row>
@@ -35884,7 +35894,7 @@
       </c>
       <c r="Z336" t="inlineStr">
         <is>
-          <t>hetzelfde getal staat als Vlaams cijfer in Tabel 26 (p.76) - zie de anomalienota; '1.149 kton voor Belgie' ook in tekst p.4</t>
+          <t>hetzelfde getal staat in Tabel 26 (p.76) in de kolom van de Vlaamse voedingssector - zie C-280, dat nu eveneens geography Belgie draagt; '1.149 kton voor Belgie' ook in tekst p.4</t>
         </is>
       </c>
     </row>
@@ -49563,7 +49573,7 @@
       </c>
       <c r="D465" t="inlineStr">
         <is>
-          <t>AGGREGAAT - Vervaardiging van plantaardige en dierlijke olien en vetten, productie hoofdstromen</t>
+          <t>AGGREGAAT - Vervaardiging van plantaardige en dierlijke olien en vetten, productie hoofdstromen (Belgisch FEDIOL-cijfer, door de bron in de Vlaamse tabel gezet)</t>
         </is>
       </c>
       <c r="E465" t="inlineStr">
@@ -49625,7 +49635,7 @@
       </c>
       <c r="U465" t="inlineStr">
         <is>
-          <t>geconsolideerde tabel verwerkingssectoren, kolom productie/hoofd; overgenomen uit Tabel 30 (FEDIOL, Belgie) maar hier als Vlaams cijfer gepresenteerd</t>
+          <t>geconsolideerde tabel verwerkingssectoren, kolom productie/hoofd; overgenomen uit Tabel 30 (FEDIOL, Belgie) maar hier als Vlaams cijfer gepresenteerd De tabeltitel zegt "Vlaamse voedingssector", maar de bron stelt zelf dat voor NACE 10.4 de FEDIOL-cijfers voor Belgie gebruikt zijn; de materiele dekking is dus Belgisch en geography staat daarom op Belgie.</t>
         </is>
       </c>
       <c r="V465" t="inlineStr">
@@ -49635,12 +49645,17 @@
       </c>
       <c r="W465" t="inlineStr">
         <is>
-          <t>Vlaanderen</t>
+          <t>Belgie</t>
         </is>
       </c>
       <c r="X465" t="inlineStr">
         <is>
           <t>read in PDF</t>
+        </is>
+      </c>
+      <c r="Z465" t="inlineStr">
+        <is>
+          <t>zelfde getal en zelfde dekking als C-518 (Tabel 30, FEDIOL Belgie, folio 115) - een herhaling in de samenvattende tabel, geen onafhankelijke meting; de reviewer kan een van beide rijen laten vervallen</t>
         </is>
       </c>
     </row>
@@ -49662,7 +49677,7 @@
       </c>
       <c r="D466" t="inlineStr">
         <is>
-          <t>AGGREGAAT - Vervaardiging van plantaardige en dierlijke olien en vetten, productie nevenstromen en productieresiduen</t>
+          <t>AGGREGAAT - Vervaardiging van plantaardige en dierlijke olien en vetten, productie nevenstromen en productieresiduen (Belgisch FEDIOL-cijfer, door de bron in de Vlaamse tabel gezet)</t>
         </is>
       </c>
       <c r="E466" t="inlineStr">
@@ -49724,7 +49739,7 @@
       </c>
       <c r="U466" t="inlineStr">
         <is>
-          <t>geconsolideerde tabel verwerkingssectoren, kolom productie/nev-res; overgenomen uit Tabel 31 (FEDIOL, Belgie) maar hier als Vlaams cijfer gepresenteerd</t>
+          <t>geconsolideerde tabel verwerkingssectoren, kolom productie/nev-res; overgenomen uit Tabel 31 (FEDIOL, Belgie) maar hier als Vlaams cijfer gepresenteerd De tabeltitel zegt "Vlaamse voedingssector", maar de bron stelt zelf dat voor NACE 10.4 de FEDIOL-cijfers voor Belgie gebruikt zijn; de materiele dekking is dus Belgisch en geography staat daarom op Belgie.</t>
         </is>
       </c>
       <c r="V466" t="inlineStr">
@@ -49734,12 +49749,17 @@
       </c>
       <c r="W466" t="inlineStr">
         <is>
-          <t>Vlaanderen</t>
+          <t>Belgie</t>
         </is>
       </c>
       <c r="X466" t="inlineStr">
         <is>
           <t>read in PDF</t>
+        </is>
+      </c>
+      <c r="Z466" t="inlineStr">
+        <is>
+          <t>zelfde getal en zelfde dekking als C-524 (Tabel 31, FEDIOL Belgie, folio 116) - een herhaling in de samenvattende tabel, geen onafhankelijke meting; de reviewer kan een van beide rijen laten vervallen</t>
         </is>
       </c>
     </row>
@@ -55406,7 +55426,7 @@
       </c>
       <c r="Z519" t="inlineStr">
         <is>
-          <t>hetzelfde getal staat als Vlaams cijfer in Tabel 28 (folio 108) - zie de anomalienota</t>
+          <t>hetzelfde getal staat in Tabel 28 (folio 108) in de kolom van de Vlaamse verwerkingssectoren - zie C-464, dat nu eveneens geography Belgie draagt</t>
         </is>
       </c>
     </row>
@@ -56055,7 +56075,7 @@
       </c>
       <c r="Z525" t="inlineStr">
         <is>
-          <t>hetzelfde getal staat als Vlaams cijfer in Tabel 28 (folio 108) - zie de anomalienota; '1.376 kton voor Belgie' ook in tekst folio 4</t>
+          <t>hetzelfde getal staat in Tabel 28 (folio 108) in de kolom van de Vlaamse verwerkingssectoren - zie C-465, dat nu eveneens geography Belgie draagt; '1.376 kton voor Belgie' ook in tekst folio 4</t>
         </is>
       </c>
     </row>

</xml_diff>